<commit_message>
Add/Update Positions.xlsx via API
</commit_message>
<xml_diff>
--- a/Positions.xlsx
+++ b/Positions.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC651"/>
+  <dimension ref="A1:AC654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50400,6 +50400,143 @@
       </c>
       <c r="AC651" t="inlineStr"/>
     </row>
+    <row r="652">
+      <c r="A652" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B652" t="n">
+        <v>0.4900347015</v>
+      </c>
+      <c r="C652" t="n">
+        <v>0.07050845850000001</v>
+      </c>
+      <c r="D652" t="inlineStr"/>
+      <c r="E652" t="inlineStr"/>
+      <c r="F652" t="inlineStr"/>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr"/>
+      <c r="I652" t="n">
+        <v>0.03704316</v>
+      </c>
+      <c r="J652" t="inlineStr"/>
+      <c r="K652" t="n">
+        <v>1597.582114482361</v>
+      </c>
+      <c r="L652" t="inlineStr"/>
+      <c r="M652" t="inlineStr"/>
+      <c r="N652" t="inlineStr"/>
+      <c r="O652" t="n">
+        <v>0.1161208636</v>
+      </c>
+      <c r="P652" t="inlineStr"/>
+      <c r="Q652" t="n">
+        <v>8.279999999999999e-07</v>
+      </c>
+      <c r="R652" t="inlineStr"/>
+      <c r="S652" t="inlineStr"/>
+      <c r="T652" t="inlineStr"/>
+      <c r="U652" t="inlineStr"/>
+      <c r="V652" t="inlineStr"/>
+      <c r="W652" t="inlineStr"/>
+      <c r="X652" t="inlineStr"/>
+      <c r="Y652" t="inlineStr"/>
+      <c r="Z652" t="n">
+        <v>32.326888690276</v>
+      </c>
+      <c r="AA652" t="n">
+        <v>0.008201770000000001</v>
+      </c>
+      <c r="AB652" t="n">
+        <v>1630.630912954237</v>
+      </c>
+      <c r="AC652" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B653" t="inlineStr"/>
+      <c r="C653" t="inlineStr"/>
+      <c r="D653" t="inlineStr"/>
+      <c r="E653" t="inlineStr"/>
+      <c r="F653" t="inlineStr"/>
+      <c r="G653" t="inlineStr"/>
+      <c r="H653" t="inlineStr"/>
+      <c r="I653" t="inlineStr"/>
+      <c r="J653" t="inlineStr"/>
+      <c r="K653" t="inlineStr"/>
+      <c r="L653" t="inlineStr"/>
+      <c r="M653" t="inlineStr"/>
+      <c r="N653" t="inlineStr"/>
+      <c r="O653" t="inlineStr"/>
+      <c r="P653" t="inlineStr"/>
+      <c r="Q653" t="inlineStr"/>
+      <c r="R653" t="inlineStr"/>
+      <c r="S653" t="inlineStr"/>
+      <c r="T653" t="inlineStr"/>
+      <c r="U653" t="inlineStr"/>
+      <c r="V653" t="inlineStr"/>
+      <c r="W653" t="inlineStr"/>
+      <c r="X653" t="inlineStr"/>
+      <c r="Y653" t="inlineStr"/>
+      <c r="Z653" t="n">
+        <v>31.162375408926</v>
+      </c>
+      <c r="AA653" t="inlineStr"/>
+      <c r="AB653" t="n">
+        <v>31.162375408926</v>
+      </c>
+      <c r="AC653" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B654" t="n">
+        <v>0.5091181</v>
+      </c>
+      <c r="C654" t="n">
+        <v>0.07207478</v>
+      </c>
+      <c r="D654" t="inlineStr"/>
+      <c r="E654" t="inlineStr"/>
+      <c r="F654" t="inlineStr"/>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr"/>
+      <c r="I654" t="n">
+        <v>0.03853640699999999</v>
+      </c>
+      <c r="J654" t="inlineStr"/>
+      <c r="K654" t="n">
+        <v>1596.443830111515</v>
+      </c>
+      <c r="L654" t="inlineStr"/>
+      <c r="M654" t="inlineStr"/>
+      <c r="N654" t="inlineStr"/>
+      <c r="O654" t="n">
+        <v>0.1190522596</v>
+      </c>
+      <c r="P654" t="inlineStr"/>
+      <c r="Q654" t="n">
+        <v>8.279999999999999e-07</v>
+      </c>
+      <c r="R654" t="inlineStr"/>
+      <c r="S654" t="inlineStr"/>
+      <c r="T654" t="inlineStr"/>
+      <c r="U654" t="inlineStr"/>
+      <c r="V654" t="inlineStr"/>
+      <c r="W654" t="inlineStr"/>
+      <c r="X654" t="inlineStr"/>
+      <c r="Y654" t="inlineStr"/>
+      <c r="Z654" t="inlineStr"/>
+      <c r="AA654" t="n">
+        <v>0.008201770000000001</v>
+      </c>
+      <c r="AB654" t="n">
+        <v>1597.190814256115</v>
+      </c>
+      <c r="AC654" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>